<commit_message>
Auto update allure report
</commit_message>
<xml_diff>
--- a/tcd-report.xlsx
+++ b/tcd-report.xlsx
@@ -50,13 +50,13 @@
     <t>User is on the login page</t>
   </si>
   <si>
-    <t>1. Enter valid username 2. Enter valid password 3. Click Login button</t>
-  </si>
-  <si>
-    <t>User should be successfully logged in and redirected to the dashboard</t>
-  </si>
-  <si>
-    <t>User was successfully logged in and redirected to the dashboard</t>
+    <t>1. Enter valid username, 2. Enter valid password, 3. Click login button</t>
+  </si>
+  <si>
+    <t>User should be redirected to the dashboard</t>
+  </si>
+  <si>
+    <t>User was successfully redirected to the dashboard</t>
   </si>
   <si>
     <t>passed</t>

</xml_diff>